<commit_message>
feat(F-NAR-009): appliquer AFF.003-02 à 09
Textes déjà fusionnés, xlsx à jour.
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.003-02.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.003-02.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:B31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Adam reprend ses affaires au parc</t>
+          <t>La pelle rouge au parc</t>
         </is>
       </c>
     </row>
@@ -602,6 +602,11 @@
           <t>secondary_lessons</t>
         </is>
       </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>AUT.RAN.001</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -830,6 +835,18 @@
       <c r="B30" t="inlineStr">
         <is>
           <t>voix-roles-v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>fil_rouge</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Au parc, le soleil baisse. Aniss reprend sa pelle rouge, sa casquette et son doudou avant de rentrer.</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1189,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Adam a joué longtemps au parc. Maman est sur le banc. Adam a une pelle rouge. Il a une casquette verte. Il a son doudou lapin. Le soleil baisse. Le banc est un peu froid. On rentre. Adam regarde encore le toboggan. On va reprendre ses affaires, avant de partir. Adam s'arrête. Il cherche la pelle près du bac. Il la prend. Il cherche la casquette sur le banc. Il la prend. Il cherche le doudou dans l'herbe. L'herbe chatouille. Il le prend. Maintenant Adam a tout. Parce qu'il a repris ses affaires, le doudou rentre aussi. Merci. Demain, les affaires seront à la maison.</t>
+          <t>Au loin, le marché sent le pain chaud. Les voix des étals montent dans la rue. Les pavés sont encore un peu humides. Dans la maison, l'écharpe d'Aniss attend sur la chaise. Aniss, on met l'écharpe ? Oui, maman. Maman noue l'écharpe. Elle est douce, un peu rêche au bord. Tu es prêt ? Oui. Ils ferment la porte. En ce moment, Aniss est au parc. Le soleil baisse derrière les arbres. Le banc est un peu froid. Maman s'assoit sur le banc. Aniss a une pelle rouge. Il a une casquette verte. Il a son doudou lapin. Le doudou est dans l'herbe. L'herbe chatouille un peu. Je fais un château, maman ! Un château ? Je regarde. Aniss verse le sable. Ça fait chh. La pelle tape le bac. Toc, toc. Un oiseau passe au-dessus. Tu as entendu l'oiseau ? Oui. Il est parti. Le ciel devient orange. Les ombres s'allongent sur le sable. Le soleil baisse, Aniss. On rentre. Encore un château ? Le château peut attendre. On reprend tes affaires, avant de partir. Aniss s'arrête. Il regarde encore le toboggan. Tu cherches la pelle ? Aniss cherche la pelle près du bac. La pelle est rouge, un peu sableuse. Il la prend. J'ai la pelle ! Bravo. Tu as repris la pelle. Et la casquette ? Aniss cherche la casquette sur le banc. Le banc est froid sous ses doigts. Il la prend. J'ai la casquette. Bien. Et le doudou ? Aniss cherche le doudou dans l'herbe. L'herbe chatouille ses mains. Il le prend. Le doudou aussi. Bravo, Aniss. Tu as repris tes affaires avant de partir. Tu as fait du bon travail. Maintenant Aniss a tout. La pelle, la casquette, le doudou. On peut rentrer. Ils marchent vers la maison. Le doudou est dans le bras d'Aniss. La pelle tape un peu sa jambe. Tu tiens bien tout ? Oui, maman.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -1312,12 +1329,75 @@
       <c r="AV2" s="2" t="inlineStr"/>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Adam a joué longtemps au parc. Maman est sur le banc. Adam a une pelle rouge. Il a une casquette verte. Il a son doudou lapin. Le soleil baisse. Le banc est un peu froid.
+          <t>narrateur|Au loin, le marché sent le pain chaud.
+narrateur|Les voix des étals montent dans la rue.
+narrateur|Les pavés sont encore un peu humides.
+narrateur|Dans la maison, l'écharpe d'Aniss attend sur la chaise.
+maman|Aniss, on met l'écharpe ?
+enfant-m|Oui, maman.
+narrateur|Maman noue l'écharpe.
+narrateur|Elle est douce, un peu rêche au bord.
+maman|Tu es prêt ?
+enfant-m|Oui.
+narrateur|Ils ferment la porte.
+narrateur|En ce moment, Aniss est au parc.
+narrateur|Le soleil baisse derrière les arbres.
+narrateur|Le banc est un peu froid.
+narrateur|Maman s'assoit sur le banc.
+narrateur|Aniss a une pelle rouge.
+narrateur|Il a une casquette verte.
+narrateur|Il a son doudou lapin.
+narrateur|Le doudou est dans l'herbe.
+narrateur|L'herbe chatouille un peu.
+enfant-m|Je fais un château, maman !
+maman|Un château ?
+maman|Je regarde.
+narrateur|Aniss verse le sable.
+narrateur|Ça fait chh.
+narrateur|La pelle tape le bac.
+narrateur|Toc, toc.
+narrateur|Un oiseau passe au-dessus.
+maman|Tu as entendu l'oiseau ?
+enfant-m|Oui.
+enfant-m|Il est parti.
+narrateur|Le ciel devient orange.
+narrateur|Les ombres s'allongent sur le sable.
+maman|Le soleil baisse, Aniss.
 maman|On rentre.
-narrateur|Adam regarde encore le toboggan.
-maman|On va reprendre ses affaires, avant de partir.
-narrateur|Adam s'arrête. Il cherche la pelle près du bac. Il la prend. Il cherche la casquette sur le banc. Il la prend. Il cherche le doudou dans l'herbe. L'herbe chatouille. Il le prend. Maintenant Adam a tout. Parce qu'il a repris ses affaires, le doudou rentre aussi.
-maman|Merci. Demain, les affaires seront à la maison.</t>
+enfant-m|Encore un château ?
+maman|Le château peut attendre.
+maman|On reprend tes affaires, avant de partir.
+narrateur|Aniss s'arrête.
+narrateur|Il regarde encore le toboggan.
+maman|Tu cherches la pelle ?
+narrateur|Aniss cherche la pelle près du bac.
+narrateur|La pelle est rouge, un peu sableuse.
+narrateur|Il la prend.
+enfant-m|J'ai la pelle !
+maman|Bravo.
+maman|Tu as repris la pelle.
+maman|Et la casquette ?
+narrateur|Aniss cherche la casquette sur le banc.
+narrateur|Le banc est froid sous ses doigts.
+narrateur|Il la prend.
+enfant-m|J'ai la casquette.
+maman|Bien.
+maman|Et le doudou ?
+narrateur|Aniss cherche le doudou dans l'herbe.
+narrateur|L'herbe chatouille ses mains.
+narrateur|Il le prend.
+enfant-m|Le doudou aussi.
+maman|Bravo, Aniss.
+maman|Tu as repris tes affaires avant de partir.
+maman|Tu as fait du bon travail.
+narrateur|Maintenant Aniss a tout.
+narrateur|La pelle, la casquette, le doudou.
+maman|On peut rentrer.
+narrateur|Ils marchent vers la maison.
+narrateur|Le doudou est dans le bras d'Aniss.
+narrateur|La pelle tape un peu sa jambe.
+maman|Tu tiens bien tout ?
+enfant-m|Oui, maman.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1349,7 +1429,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Avant de partir du parc, que fait Adam ?</t>
+          <t>Avant de partir du parc, que fait Aniss ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -1509,7 +1589,7 @@
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Avant de partir du parc, que fait Adam ?</t>
+          <t>narrateur|Avant de partir du parc, que fait Aniss ?</t>
         </is>
       </c>
       <c r="AX3" t="inlineStr">
@@ -1541,7 +1621,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Adam a cherché. Il a repris la pelle, la casquette, le doudou. C'était avant de partir. Les affaires rentrent à la maison.</t>
+          <t>Aniss a cherché. Il a repris la pelle. Il a repris la casquette. Il a repris le doudou. C'était avant de partir. Tu as tout, Aniss ? Oui. J'ai tout. Bravo. Les affaires rentrent à la maison. Le doudou rentre aussi.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -1685,10 +1765,19 @@
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Adam a cherché. Il a repris la pelle, la casquette, le doudou. C'était avant de partir. Les affaires rentrent à la maison.</t>
-        </is>
-      </c>
-      <c r="AX4" t="inlineStr"/>
+          <t>narrateur|Aniss a cherché.
+narrateur|Il a repris la pelle.
+narrateur|Il a repris la casquette.
+narrateur|Il a repris le doudou.
+narrateur|C'était avant de partir.
+maman|Tu as tout, Aniss ?
+enfant-m|Oui.
+enfant-m|J'ai tout.
+maman|Bravo.
+maman|Les affaires rentrent à la maison.
+narrateur|Le doudou rentre aussi.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1713,7 +1802,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Adam marche près de maman. Le doudou est dans son bras. La pelle tape un peu.</t>
+          <t>Aniss marche près de maman. La rue sent encore le marché. Le pain est loin, maintenant. Ils arrivent à la porte. Tu poses la pelle près des chaussures ? Aniss pose la pelle. Il pose la casquette. Le doudou reste dans son bras. Merci. Demain, les affaires seront à la maison. Demain, au parc encore ? Demain, on verra. Tu as repris tes affaires avant de partir. La maison est calme. L'écharpe retrouve la chaise.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1849,10 +1938,23 @@
       <c r="AV5" s="2" t="inlineStr"/>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Adam marche près de maman. Le doudou est dans son bras. La pelle tape un peu.</t>
-        </is>
-      </c>
-      <c r="AX5" t="inlineStr"/>
+          <t>narrateur|Aniss marche près de maman.
+narrateur|La rue sent encore le marché.
+narrateur|Le pain est loin, maintenant.
+narrateur|Ils arrivent à la porte.
+maman|Tu poses la pelle près des chaussures ?
+narrateur|Aniss pose la pelle.
+narrateur|Il pose la casquette.
+narrateur|Le doudou reste dans son bras.
+maman|Merci.
+maman|Demain, les affaires seront à la maison.
+enfant-m|Demain, au parc encore ?
+maman|Demain, on verra.
+maman|Tu as repris tes affaires avant de partir.
+narrateur|La maison est calme.
+narrateur|L'écharpe retrouve la chaise.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1877,7 +1979,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>L'histoire est finie.</t>
+          <t>J'ai repris mes affaires. Avant de partir. Bravo, Aniss. Tu as fait du bon travail. L'histoire est finie.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -2017,10 +2119,13 @@
       <c r="AV6" s="2" t="inlineStr"/>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|L'histoire est finie.</t>
-        </is>
-      </c>
-      <c r="AX6" t="inlineStr"/>
+          <t>enfant-m|J'ai repris mes affaires.
+maman|Avant de partir.
+maman|Bravo, Aniss.
+maman|Tu as fait du bon travail.
+narrateur|L'histoire est finie.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:AV6"/>
@@ -2039,7 +2144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2077,6 +2182,13 @@
       <c r="A5" t="inlineStr">
         <is>
           <t>F-AUD-007 colonne sons ; vide = silence ; jamais parler dans le bruit</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>F-NAR-009 ouverture du monde, fusion agents</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(F-NAR-019): ATOM-AUT.AFF.003-02 La maison du lapin
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.003-02.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.003-02.xlsx
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Aniss veut une maison avec une porte pour son lapin. Au parc, le soleil baisse. Il reprend pelle, casquette et lapin pour finir la porte à la maison.</t>
+          <t>Aniss connaît la cuisine. Un éclat d'orange cligne sur le bois. Il veut la maison du lapin, maintenant. Au parc, il pousse le doudou dans un tas trop mou : le lapin glisse dans l'herbe. Il part les mains vides, refuse, reprend pelle, casquette, lapin. À la cuisine, l'oreille se coince. Il refuse de foncer, suit l'éclat, plie une porte. Le lapin rentre. L'éclat reste pâle sur le bois.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Sur la table, les peaux d'orange brillent. Elles sentent encore le goûter. Un peu de jus a collé au bois. Tes doigts sont collants, Aniss. Ça sent l'orange. Maman passe un linge tiède. Le linge est doux, un peu rêche. On va au parc ? Oui. Avec le lapin. Le doudou lapin attend près de la porte. Sa grande oreille plie un peu. Ils ferment la porte. La rue sent encore l'orange, un peu. En ce moment, Aniss est au parc. Le soleil baisse derrière les arbres. Le banc est un peu froid. Maman s'assoit. Aniss a une pelle rouge. Il a une casquette verte. Le lapin est dans l'herbe. Je lui fais une maison. Une maison pour le lapin ? Oui. Avec une porte. Aniss verse le sable. Ça fait chh. La pelle tape le bac. Toc, toc. Les murs du château montent. Le lapin regarde, dans l'herbe. L'herbe chatouille un peu. Tu as entendu l'oiseau ? Oui. Il est parti. Le ciel devient orange. Comme les peaux, sur la table. Le soleil baisse, Aniss. On rentre. La porte n'est pas finie. Le château reste ici. La porte, on la fera à la maison. Avec la pelle ? Avec la pelle. Et le lapin. On reprend ses affaires, avant de partir. Aniss s'arrête. Il regarde ses mains. Elles sont vides. La pelle est encore dans le sable. Il la prend. Un peu de sable tombe. J'ai la pelle. Bien. Elle servira pour la porte. La casquette est sur le banc. Le lapin est encore dans l'herbe. Aniss cherche des yeux.</t>
+          <t>La lumière baisse sur les carreaux de la cuisine. Aniss connaît cette table, le bol, la porte. La fenêtre est tiède, un peu. Un détail paraît nouveau, sur le bois. Après le goûter, un éclat d'orange cligne. Le jus a attrapé le soleil, bas. Aniss, tu vois l'éclat ? Il brille, maman. Je veux la maison du lapin, maintenant ! Le doudou lapin attend près de la porte. Sa grande oreille plie un peu. La pelle rouge est contre le mur. La casquette verte pend au crochet. On va au parc ? Oui. Avec une porte, pour lui. Maman passe un linge tiède sur ses doigts. Les doigts étaient collants, un peu. Ils ferment la porte. La rue sent l'orange, tiède. En ce moment, Aniss court vers le banc du parc. Le soleil baisse derrière les arbres. Le banc est froid, un peu. Maman s'assoit. Aniss pose le lapin dans l'herbe. Sa maison, tout de suite. Il verse du sable avec la pelle rouge. Ça fait chh, trop vite. Les murs tombent, mous. Reste là ! Il pousse le lapin dans le tas. Le lapin glisse, sans un bruit. Il roule dans l'herbe, oreille pliée. Oh. Il est parti ! Le sourire d'Aniss disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Maman s'accroupit à sa hauteur. Tu le cherches, Aniss ? Il ne veut pas rentrer. Le soleil baisse. On rentre. La porte n'est pas finie. La maison, on la fera à la maison. Avec la pelle ? Avec la pelle. Et le lapin. Aniss veut partir d'un coup. Il marche vers la grille, les mains vides. La pelle reste dans le sable. La casquette reste sur le banc. Le lapin reste dans l'herbe. Mes mains sont vides. Tu regardes tes affaires ?</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Sur la table, les peaux d'orange brillent. Elles sentent encore le goûter. Un peu de jus a collé au bois. Tes doigts sont collants, Aniss. Ça sent l'orange. Maman passe un linge tiède. Le linge est doux, un peu rêche. On va au parc ? Oui. Avec le lapin. Le doudou lapin attend près de la porte. Sa grande oreille plie un peu. Ils ferment la porte. La rue sent encore l'orange, un peu. En ce moment, Aniss est au parc. Le soleil baisse derrière les arbres. Le banc est un peu froid. Maman s'assoit. Aniss a une pelle rouge. Il a une casquette verte. Le lapin est dans l'herbe. Je lui fais une maison. Une maison pour le lapin ? Oui. Avec une porte. Aniss verse le sable. Ça fait chh. La pelle tape le bac. Toc, toc. Les murs du château montent. Le lapin regarde, dans l'herbe. L'herbe chatouille un peu. Tu as entendu l'oiseau ? Oui. Il est parti. Le ciel devient orange. Comme les peaux, sur la table. Le soleil baisse, Aniss. On rentre. La porte n'est pas finie. Le château reste ici. La porte, on la fera à la maison. Avec la pelle ? Avec la pelle. Et le lapin. On reprend ses affaires, avant de partir. Aniss s'arrête. Il regarde ses mains. Elles sont vides. La pelle est encore dans le sable. Il la prend. Un peu de sable tombe. J'ai la pelle. Bien. Elle servira pour la porte. La casquette est sur le banc. Le lapin est encore dans l'herbe. Aniss cherche des yeux.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La lumière baisse sur les carreaux de la cuisine. Aniss connaît cette table, le bol, la porte. La fenêtre est tiède, un peu. Un détail paraît nouveau, sur le bois. Après le goûter, un &lt;emphasis level="moderate"&gt;éclat d'orange&lt;/emphasis&gt; cligne. Le jus a attrapé le soleil, bas. Aniss, tu vois l'éclat ? Il brille, maman. Je veux la maison du lapin, maintenant ! Le doudou lapin attend près de la porte. Sa grande oreille plie un peu. La pelle rouge est contre le mur. La casquette verte pend au crochet. On va au parc ? Oui. Avec une porte, pour lui. Maman passe un linge tiède sur ses doigts. Les doigts étaient collants, un peu. Ils ferment la porte. La rue sent l'orange, tiède. En ce moment, Aniss court vers le banc du parc. Le soleil baisse derrière les arbres. Le banc est froid, un peu. Maman s'assoit. Aniss pose le lapin dans l'herbe. Sa maison, tout de suite. Il verse du sable avec la pelle rouge. Ça fait chh, trop vite. Les murs tombent, mous. Reste là ! Il pousse le lapin dans le tas. Le lapin glisse, sans un bruit. Il roule dans l'herbe, oreille pliée. Oh. Il est parti ! Le sourire d'Aniss disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Maman s'accroupit à sa hauteur. Tu le cherches, Aniss ? Il ne veut pas rentrer. Le soleil baisse. On rentre. La porte n'est pas finie. La maison, on la fera à la maison. Avec la pelle ? Avec la pelle. Et le lapin. Aniss veut partir d'un coup. Il marche vers la grille, les mains vides. La pelle reste dans le sable. La casquette reste sur le banc. Le lapin reste dans l'herbe. Mes mains sont vides. Tu regardes tes affaires ?&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Adam a joué longtemps au parc. Maman est sur le banc. Adam a une pelle rouge. Il a une casquette verte. Il a son doudou lapin. Le soleil baisse. Le banc est un peu froid. Maman dit : on rentre. Adam regarde encore le toboggan. Maman dit : on va &lt;emphasis&gt;reprendre&lt;/emphasis&gt; ses affaires, avant de partir. Adam s'arrête. Il cherche la pelle près du bac. Il la prend. Il cherche la casquette sur le banc. Il la prend. Il cherche le doudou dans l'herbe. L'herbe chatouille. Il le prend. Maintenant Adam a tout. Parce qu'il a repris ses affaires, le doudou rentre aussi. Maman dit : merci. Demain, les affaires seront à la maison. [pause]</t>
+          <t>La lumière baisse sur les carreaux de la cuisine. Aniss connaît cette table, le bol, la porte. La fenêtre est tiède, un peu. Un détail paraît nouveau, sur le bois. Après le goûter, un &lt;emphasis&gt;éclat d'orange&lt;/emphasis&gt; cligne. Le jus a attrapé le soleil, bas. Aniss, tu vois l'éclat ? Il brille, maman. Je veux la maison du lapin, maintenant ! Le doudou lapin attend près de la porte. Sa grande oreille plie un peu. La pelle rouge est contre le mur. La casquette verte pend au crochet. On va au parc ? Oui. Avec une porte, pour lui. Maman passe un linge tiède sur ses doigts. Les doigts étaient collants, un peu. Ils ferment la porte. La rue sent l'orange, tiède. En ce moment, Aniss court vers le banc du parc. Le soleil baisse derrière les arbres. Le banc est froid, un peu. Maman s'assoit. Aniss pose le lapin dans l'herbe. Sa maison, tout de suite. Il verse du sable avec la pelle rouge. Ça fait chh, trop vite. Les murs tombent, mous. Reste là ! Il pousse le lapin dans le tas. Le lapin glisse, sans un bruit. Il roule dans l'herbe, oreille pliée. Oh. Il est parti ! Le sourire d'Aniss disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Maman s'accroupit à sa hauteur. Tu le cherches, Aniss ? Il ne veut pas rentrer. Le soleil baisse. On rentre. La porte n'est pas finie. La maison, on la fera à la maison. Avec la pelle ? Avec la pelle. Et le lapin. Aniss veut partir d'un coup. Il marche vers la grille, les mains vides. La pelle reste dans le sable. La casquette reste sur le banc. Le lapin reste dans l'herbe. Mes mains sont vides. Tu regardes tes affaires ? [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1280,30 +1280,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>reprendre</t>
+          <t>éclat d'orange</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1326,72 +1326,72 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience_curieuse puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_la_maison_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Sur la table, les peaux d'orange brillent.
-narrateur|Elles sentent encore le goûter.
-narrateur|Un peu de jus a collé au bois.
-maman|Tes doigts sont collants, Aniss.
-enfant-m|Ça sent l'orange.
-narrateur|Maman passe un linge tiède.
-narrateur|Le linge est doux, un peu rêche.
+          <t>narrateur|La lumière baisse sur les carreaux de la cuisine.
+narrateur|Aniss connaît cette table, le bol, la porte.
+narrateur|La fenêtre est tiède, un peu.
+narrateur|Un détail paraît nouveau, sur le bois.
+narrateur|Après le goûter, un éclat d'orange cligne.
+narrateur|Le jus a attrapé le soleil, bas.
+maman|Aniss, tu vois l'éclat ?
+enfant-m|Il brille, maman.
+enfant-m|Je veux la maison du lapin, maintenant !
+narrateur|Le doudou lapin attend près de la porte.
+narrateur|Sa grande oreille plie un peu.
+narrateur|La pelle rouge est contre le mur.
+narrateur|La casquette verte pend au crochet.
 maman|On va au parc ?
 enfant-m|Oui.
-enfant-m|Avec le lapin.
-narrateur|Le doudou lapin attend près de la porte.
-narrateur|Sa grande oreille plie un peu.
+enfant-m|Avec une porte, pour lui.
+narrateur|Maman passe un linge tiède sur ses doigts.
+narrateur|Les doigts étaient collants, un peu.
 narrateur|Ils ferment la porte.
-narrateur|La rue sent encore l'orange, un peu.
-narrateur|En ce moment, Aniss est au parc.
+narrateur|La rue sent l'orange, tiède.
+narrateur|En ce moment, Aniss court vers le banc du parc.
 narrateur|Le soleil baisse derrière les arbres.
-narrateur|Le banc est un peu froid.
+narrateur|Le banc est froid, un peu.
 narrateur|Maman s'assoit.
-narrateur|Aniss a une pelle rouge.
-narrateur|Il a une casquette verte.
-narrateur|Le lapin est dans l'herbe.
-enfant-m|Je lui fais une maison.
-maman|Une maison pour le lapin ?
-enfant-m|Oui.
-enfant-m|Avec une porte.
-narrateur|Aniss verse le sable.
-narrateur|Ça fait chh.
-narrateur|La pelle tape le bac.
-narrateur|Toc, toc.
-narrateur|Les murs du château montent.
-narrateur|Le lapin regarde, dans l'herbe.
-narrateur|L'herbe chatouille un peu.
-maman|Tu as entendu l'oiseau ?
-enfant-m|Oui.
-enfant-m|Il est parti.
-narrateur|Le ciel devient orange.
-narrateur|Comme les peaux, sur la table.
-maman|Le soleil baisse, Aniss.
+narrateur|Aniss pose le lapin dans l'herbe.
+enfant-m|Sa maison, tout de suite.
+narrateur|Il verse du sable avec la pelle rouge.
+narrateur|Ça fait chh, trop vite.
+narrateur|Les murs tombent, mous.
+enfant-m|Reste là !
+narrateur|Il pousse le lapin dans le tas.
+narrateur|Le lapin glisse, sans un bruit.
+narrateur|Il roule dans l'herbe, oreille pliée.
+enfant-m|Oh.
+enfant-m|Il est parti !
+narrateur|Le sourire d'Aniss disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Maman s'accroupit à sa hauteur.
+maman|Tu le cherches, Aniss ?
+enfant-m|Il ne veut pas rentrer.
+maman|Le soleil baisse.
 maman|On rentre.
 enfant-m|La porte n'est pas finie.
-maman|Le château reste ici.
-maman|La porte, on la fera à la maison.
+maman|La maison, on la fera à la maison.
 enfant-m|Avec la pelle ?
 maman|Avec la pelle.
 maman|Et le lapin.
-maman|On reprend ses affaires, avant de partir.
-narrateur|Aniss s'arrête.
-narrateur|Il regarde ses mains.
-narrateur|Elles sont vides.
-narrateur|La pelle est encore dans le sable.
-narrateur|Il la prend.
-narrateur|Un peu de sable tombe.
-enfant-m|J'ai la pelle.
-maman|Bien.
-maman|Elle servira pour la porte.
-narrateur|La casquette est sur le banc.
-narrateur|Le lapin est encore dans l'herbe.
-narrateur|Aniss cherche des yeux.</t>
+narrateur|Aniss veut partir d'un coup.
+narrateur|Il marche vers la grille, les mains vides.
+narrateur|La pelle reste dans le sable.
+narrateur|La casquette reste sur le banc.
+narrateur|Le lapin reste dans l'herbe.
+enfant-m|Mes mains sont vides.
+maman|Tu regardes tes affaires ?</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
         <is>
-          <t>enfants_parc</t>
+          <t>porte,enfants_parc</t>
         </is>
       </c>
     </row>
@@ -1418,17 +1418,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Avant de partir, que fait Aniss ?</t>
+          <t>Aniss prépare le retour. Ses affaires attendent au parc. Avant de partir, que fait Aniss ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Avant de partir, que fait Aniss ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Aniss prépare le retour. Ses &lt;emphasis level="moderate"&gt;affaires&lt;/emphasis&gt; attendent au parc. Avant de partir, que fait Aniss ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;&lt;emphasis&gt;avant&lt;/emphasis&gt; de partir du parc, que fait Adam ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Aniss prépare le retour. Ses &lt;emphasis&gt;affaires&lt;/emphasis&gt; attendent au parc. Avant de partir, que fait Aniss ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1491,7 +1491,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1502,7 +1502,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1517,38 +1517,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
-          <t>avant</t>
+          <t>affaires</t>
         </is>
       </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1563,22 +1563,24 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=avant_de_partir_il_reprend; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Avant de partir, que fait Aniss ?</t>
+          <t>narrateur|Aniss prépare le retour.
+narrateur|Ses affaires attendent au parc.
+narrateur|Avant de partir, que fait Aniss ?</t>
         </is>
       </c>
       <c r="AX3" t="inlineStr">
@@ -1610,17 +1612,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Aniss cherche la casquette. Le banc est froid sous ses doigts. La casquette est sous la main de maman. Oh. Je la cachais. Ma casquette ! Il la prend. Il va dans l'herbe. L'herbe chatouille. Le lapin a une oreille pliée. Le voilà. Aniss le prend contre lui. Tu as repris tes affaires. Avant de partir. Oui. On peut aller faire la porte. Ils marchent vers la maison. La pelle tape un peu sa jambe. Tu tiens bien tout ? Oui, maman.</t>
+          <t>Aniss refuse de partir les mains vides. Il revient vers le tas de sable. La pelle rouge attend, couchée. Il la reprend. Un peu de sable tombe. J'ai la pelle. Il va vers le banc froid. La casquette verte est sous la main de maman. Je la tenais. Ma casquette ! Il la prend, verte, un peu froide. Il va dans l'herbe. L'herbe chatouille un peu. Le lapin a une oreille pliée. Le voilà. Aniss le prend contre lui. Merci, Aniss. Tu tiens bien tout ? Oui, maman. Ils marchent vers la maison. La pelle tape un peu sa jambe. On va faire la porte. Oui. On ouvre la cuisine ? Oui.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Aniss cherche la casquette. Le banc est froid sous ses doigts. La casquette est sous la main de maman. Oh. Je la cachais. Ma casquette ! Il la prend. Il va dans l'herbe. L'herbe chatouille. Le lapin a une oreille pliée. Le voilà. Aniss le prend contre lui. Tu as repris tes affaires. Avant de partir. Oui. On peut aller faire la porte. Ils marchent vers la maison. La pelle tape un peu sa jambe. Tu tiens bien tout ? Oui, maman.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Aniss refuse de partir les mains vides. Il revient vers le tas de sable. La &lt;emphasis level="moderate"&gt;pelle&lt;/emphasis&gt; rouge attend, couchée. Il la reprend. Un peu de sable tombe. J'ai la pelle. Il va vers le banc froid. La casquette verte est sous la main de maman. Je la tenais. Ma casquette ! Il la prend, verte, un peu froide. Il va dans l'herbe. L'herbe chatouille un peu. Le lapin a une oreille pliée. Le voilà. Aniss le prend contre lui. Merci, Aniss. Tu tiens bien tout ? Oui, maman. Ils marchent vers la maison. La pelle tape un peu sa jambe. On va faire la porte. Oui. On ouvre la cuisine ? Oui.&lt;/prosody&gt;&lt;break time="450ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Adam a cherché. Il a repris la pelle, la casquette, le doudou. C'était &lt;emphasis&gt;avant&lt;/emphasis&gt; de partir. Les affaires rentrent à la maison. [pause]</t>
+          <t>Aniss refuse de partir les mains vides. Il revient vers le tas de sable. La &lt;emphasis&gt;pelle&lt;/emphasis&gt; rouge attend, couchée. Il la reprend. Un peu de sable tombe. J'ai la pelle. Il va vers le banc froid. La casquette verte est sous la main de maman. Je la tenais. Ma casquette ! Il la prend, verte, un peu froide. Il va dans l'herbe. L'herbe chatouille un peu. Le lapin a une oreille pliée. Le voilà. Aniss le prend contre lui. Merci, Aniss. Tu tiens bien tout ? Oui, maman. Ils marchent vers la maison. La pelle tape un peu sa jambe. On va faire la porte. Oui. On ouvre la cuisine ? Oui. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1678,7 +1680,7 @@
         <v>0.92</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.2</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1701,7 +1703,7 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>avant</t>
+          <t>pelle</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
@@ -1715,16 +1717,16 @@
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1749,31 +1751,41 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=confirmation; intention=relancer; emotion=fierté_calme; intensite=1; destinataire=enfant; sous_texte=il_reprend_sans_foncer; tempo=naturel; sourire=léger; respiration=fluide</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Aniss cherche la casquette.
-narrateur|Le banc est froid sous ses doigts.
-narrateur|La casquette est sous la main de maman.
-maman|Oh.
-maman|Je la cachais.
+          <t>narrateur|Aniss refuse de partir les mains vides.
+narrateur|Il revient vers le tas de sable.
+narrateur|La pelle rouge attend, couchée.
+narrateur|Il la reprend.
+narrateur|Un peu de sable tombe.
+enfant-m|J'ai la pelle.
+narrateur|Il va vers le banc froid.
+narrateur|La casquette verte est sous la main de maman.
+maman|Je la tenais.
 enfant-m|Ma casquette !
-narrateur|Il la prend.
+narrateur|Il la prend, verte, un peu froide.
 narrateur|Il va dans l'herbe.
-narrateur|L'herbe chatouille.
+narrateur|L'herbe chatouille un peu.
 narrateur|Le lapin a une oreille pliée.
 enfant-m|Le voilà.
 narrateur|Aniss le prend contre lui.
-maman|Tu as repris tes affaires.
-enfant-m|Avant de partir.
-maman|Oui.
-maman|On peut aller faire la porte.
+maman|Merci, Aniss.
+maman|Tu tiens bien tout ?
+enfant-m|Oui, maman.
 narrateur|Ils marchent vers la maison.
 narrateur|La pelle tape un peu sa jambe.
-maman|Tu tiens bien tout ?
-enfant-m|Oui, maman.</t>
+enfant-m|On va faire la porte.
+maman|Oui.
+maman|On ouvre la cuisine ?
+enfant-m|Oui.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>pelle,porte</t>
         </is>
       </c>
     </row>
@@ -1800,17 +1812,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Ils arrivent à la porte. Les peaux d'orange sont encore sur la table. Elles ont attendu. Oui. Comme le lapin. Tu poses la pelle près des chaussures ? Aniss pose la pelle. Il pose la casquette. Le lapin reste dans son bras. Maman sort une boîte. Une petite boîte à chaussures. Voici la maison. Et la porte ? On plie un bout. Ça fait une porte. Aniss plie le carton. Ça fait un petit clap. Il glisse le lapin dedans. Il rentre. Sa maison est prête. Aniss souffle un peu, tout doux. Il dort. Bravo. Tu as trouvé le lapin.</t>
+          <t>Ils arrivent dans la cuisine. Sur le bois, l'éclat d'orange cligne, pâle. Il a attendu. Oui. Comme le lapin. Tu poses la pelle près des chaussures ? Aniss pose la pelle. Il pose la casquette. Le lapin reste dans son bras. Maman sort une boîte à chaussures. Voici la maison. Et la porte, maintenant ! Il veut glisser le lapin, d'un coup. L'oreille se coince au bord. Ça ne rentre pas ! Le carton refuse, dur. Aniss veut pousser plus fort. Cette fois, il refuse de foncer. Attends, je regarde. Personne ne donne la réponse. Il observe la boîte, puis la cuisine. Sur le bois, l'éclat d'orange cligne. C'est celui du goûter. Tu le vois, sur la table ? Oui, il montre un pli. L'éclat d'orange allume une ligne sur le carton. Aniss plie ce bout, sans brusquer. Ça fait un petit clap. Une porte s'ouvre, nette. Il glisse le lapin par la porte. Il rentre. Sa maison est prête ? Oui, maman.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Ils arrivent à la porte. Les peaux d'orange sont encore sur la table. Elles ont attendu. Oui. Comme le lapin. Tu poses la pelle près des chaussures ? Aniss pose la pelle. Il pose la casquette. Le lapin reste dans son bras. Maman sort une boîte. Une petite boîte à chaussures. Voici la maison. Et la porte ? On plie un bout. Ça fait une porte. Aniss plie le carton. Ça fait un petit clap. Il glisse le lapin dedans. Il rentre. Sa maison est prête. Aniss souffle un peu, tout doux. Il dort. Bravo. Tu as trouvé le lapin.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Ils arrivent dans la cuisine. Sur le bois, l'&lt;emphasis level="moderate"&gt;éclat d'orange&lt;/emphasis&gt; cligne, pâle. Il a attendu. Oui. Comme le lapin. Tu poses la pelle près des chaussures ? Aniss pose la pelle. Il pose la casquette. Le lapin reste dans son bras. Maman sort une boîte à chaussures. Voici la maison. Et la porte, maintenant ! Il veut glisser le lapin, d'un coup. L'oreille se coince au bord. Ça ne rentre pas ! Le carton refuse, dur. Aniss veut pousser plus fort. Cette fois, il refuse de foncer. Attends, je regarde. Personne ne donne la réponse. Il observe la boîte, puis la cuisine. Sur le bois, l'éclat d'orange cligne. C'est celui du goûter. Tu le vois, sur la table ? Oui, il montre un pli. L'éclat d'orange allume une ligne sur le carton. Aniss plie ce bout, sans brusquer. Ça fait un petit clap. Une porte s'ouvre, nette. Il glisse le lapin par la porte. Il rentre. Sa maison est prête ? Oui, maman.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Adam marche près de maman. Le doudou est dans son bras. La pelle tape un peu. [pause]</t>
+          <t>&lt;low-pitch&gt;Ils arrivent dans la cuisine. Sur le bois, l'&lt;emphasis&gt;éclat d'orange&lt;/emphasis&gt; cligne, pâle. Il a attendu. Oui. Comme le lapin. Tu poses la pelle près des chaussures ? Aniss pose la pelle. Il pose la casquette. Le lapin reste dans son bras. Maman sort une boîte à chaussures. Voici la maison. Et la porte, maintenant ! Il veut glisser le lapin, d'un coup. L'oreille se coince au bord. Ça ne rentre pas ! Le carton refuse, dur. Aniss veut pousser plus fort. Cette fois, il refuse de foncer. Attends, je regarde. Personne ne donne la réponse. Il observe la boîte, puis la cuisine. Sur le bois, l'éclat d'orange cligne. C'est celui du goûter. Tu le vois, sur la table ? Oui, il montre un pli. L'éclat d'orange allume une ligne sur le carton. Aniss plie ce bout, sans brusquer. Ça fait un petit clap. Une porte s'ouvre, nette. Il glisse le lapin par la porte. Il rentre. Sa maison est prête ? Oui, maman.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1857,7 +1869,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1865,22 +1877,26 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
         <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1889,28 +1905,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat d'orange</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1919,47 +1939,65 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_retrouve_l_eclat; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Ils arrivent à la porte.
-narrateur|Les peaux d'orange sont encore sur la table.
-enfant-m|Elles ont attendu.
+          <t>narrateur|Ils arrivent dans la cuisine.
+narrateur|Sur le bois, l'éclat d'orange cligne, pâle.
+enfant-m|Il a attendu.
 maman|Oui.
 maman|Comme le lapin.
 maman|Tu poses la pelle près des chaussures ?
 narrateur|Aniss pose la pelle.
 narrateur|Il pose la casquette.
 narrateur|Le lapin reste dans son bras.
-narrateur|Maman sort une boîte.
-narrateur|Une petite boîte à chaussures.
+narrateur|Maman sort une boîte à chaussures.
 maman|Voici la maison.
-enfant-m|Et la porte ?
-maman|On plie un bout.
-maman|Ça fait une porte.
-narrateur|Aniss plie le carton.
+enfant-m|Et la porte, maintenant !
+narrateur|Il veut glisser le lapin, d'un coup.
+narrateur|L'oreille se coince au bord.
+enfant-m|Ça ne rentre pas !
+narrateur|Le carton refuse, dur.
+narrateur|Aniss veut pousser plus fort.
+narrateur|Cette fois, il refuse de foncer.
+enfant-m|Attends, je regarde.
+narrateur|Personne ne donne la réponse.
+narrateur|Il observe la boîte, puis la cuisine.
+narrateur|Sur le bois, l'éclat d'orange cligne.
+enfant-m|C'est celui du goûter.
+maman|Tu le vois, sur la table ?
+enfant-m|Oui, il montre un pli.
+narrateur|L'éclat d'orange allume une ligne sur le carton.
+narrateur|Aniss plie ce bout, sans brusquer.
 narrateur|Ça fait un petit clap.
-narrateur|Il glisse le lapin dedans.
+narrateur|Une porte s'ouvre, nette.
+narrateur|Il glisse le lapin par la porte.
 enfant-m|Il rentre.
-maman|Sa maison est prête.
-narrateur|Aniss souffle un peu, tout doux.
-enfant-m|Il dort.
-maman|Bravo.
-maman|Tu as trouvé le lapin.</t>
+maman|Sa maison est prête ?
+enfant-m|Oui, maman.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>carton,porte</t>
         </is>
       </c>
     </row>
@@ -1986,17 +2024,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le lapin a sa maison. Et toi, tu as repris tes affaires. La pelle repose près des chaussures. L'orange sent encore un peu.</t>
+          <t>Ils restent un moment, sans parler. Le lapin est dans sa maison. Il a sa porte. Tu as posé la pelle ? Oui, près des chaussures. La casquette repose au crochet. L'éclat d'orange reste, pâle, sur le bois.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le lapin a sa maison. Et toi, tu as repris tes affaires. La pelle repose près des chaussures. L'orange sent encore un peu.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent un moment, sans parler. Le lapin est dans sa maison. Il a sa porte. Tu as posé la pelle ? Oui, près des chaussures. La casquette repose au crochet. L'&lt;emphasis level="moderate"&gt;éclat d'orange&lt;/emphasis&gt; reste, pâle, sur le bois.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent un moment, sans parler. Le lapin est dans sa maison. Il a sa porte. Tu as posé la pelle ? Oui, près des chaussures. La casquette repose au crochet. L'&lt;emphasis&gt;éclat d'orange&lt;/emphasis&gt; reste, pâle, sur le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2043,7 +2081,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2051,10 +2089,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2063,12 +2101,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2077,17 +2115,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat d'orange</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2096,11 +2138,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2109,27 +2151,39 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_reste_pale_sur_le_bois; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-m|Le lapin a sa maison.
-maman|Et toi, tu as repris tes affaires.
-narrateur|La pelle repose près des chaussures.
-narrateur|L'orange sent encore un peu.</t>
+          <t>narrateur|Ils restent un moment, sans parler.
+narrateur|Le lapin est dans sa maison.
+enfant-m|Il a sa porte.
+maman|Tu as posé la pelle ?
+enfant-m|Oui, près des chaussures.
+narrateur|La casquette repose au crochet.
+narrateur|L'éclat d'orange reste, pâle, sur le bois.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>porte</t>
         </is>
       </c>
     </row>
@@ -2150,7 +2204,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2242,6 +2296,13 @@
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>